<commit_message>
[Fix] 재시작 시 _currentSpecialEventStep 미초기화 버그 수정
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/CBASpecialEvent.xlsx
+++ b/JsonConverter/ExcelFiles/CBASpecialEvent.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GameProjects\CBA\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49A69B5A-A555-4D40-B746-E4C494292EA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22D582F9-937A-406C-811F-3C6080C3C6CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -127,9 +127,6 @@
   </si>
   <si>
     <t>Bee</t>
-  </si>
-  <si>
-    <t>네놈의 꿀을 내놔라!</t>
   </si>
   <si>
     <t>BG_Forest</t>
@@ -393,12 +390,108 @@
     </r>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>야</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>뚱곰</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">! </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>꿀</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>내놔</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">! </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>촤핫</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>!</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>\n넌 살 좀 빼야돼~</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -442,6 +535,17 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial Unicode MS"/>
       <family val="3"/>
       <charset val="129"/>
     </font>
@@ -506,7 +610,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -530,6 +634,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -835,7 +942,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O19"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
@@ -850,7 +957,7 @@
     <col min="15" max="15" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="21.95" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -897,7 +1004,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" ht="18" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
@@ -944,7 +1051,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" ht="21.95" customHeight="1">
       <c r="A3" s="3" t="s">
         <v>17</v>
       </c>
@@ -991,7 +1098,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="39.950000000000003" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>32</v>
       </c>
@@ -1002,43 +1109,43 @@
         <v>1</v>
       </c>
       <c r="D4" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="H4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="I4" s="5" t="s">
         <v>37</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>38</v>
       </c>
       <c r="J4" s="5">
         <v>60</v>
       </c>
       <c r="K4" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="L4" s="5" t="s">
-        <v>40</v>
-      </c>
       <c r="M4" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="N4" s="5">
         <v>40</v>
       </c>
       <c r="O4" s="5"/>
     </row>
-    <row r="5" spans="1:15" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="39.950000000000003" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>33</v>
@@ -1047,41 +1154,41 @@
         <v>2</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="F5" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="G5" s="5" t="s">
+      <c r="H5" s="5" t="s">
         <v>43</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>44</v>
       </c>
       <c r="I5" s="5"/>
       <c r="J5" s="5">
         <v>70</v>
       </c>
       <c r="K5" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="M5" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="L5" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="M5" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="N5" s="5">
         <v>50</v>
       </c>
       <c r="O5" s="5"/>
     </row>
-    <row r="6" spans="1:15" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="39.950000000000003" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>33</v>
@@ -1090,31 +1197,31 @@
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="F6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>49</v>
-      </c>
       <c r="H6" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J6" s="5">
         <v>40</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M6" s="5"/>
       <c r="N6" s="5">
@@ -1122,9 +1229,9 @@
       </c>
       <c r="O6" s="5"/>
     </row>
-    <row r="7" spans="1:15" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" ht="39.950000000000003" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>33</v>
@@ -1133,43 +1240,43 @@
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="F7" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="F7" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>53</v>
-      </c>
       <c r="H7" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J7" s="5">
         <v>65</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L7" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N7" s="5">
         <v>50</v>
       </c>
       <c r="O7" s="5"/>
     </row>
-    <row r="8" spans="1:15" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="39.950000000000003" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>33</v>
@@ -1178,13 +1285,13 @@
         <v>3</v>
       </c>
       <c r="D8" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>56</v>
-      </c>
       <c r="F8" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G8" s="5"/>
       <c r="H8" s="5"/>
@@ -1199,12 +1306,12 @@
         <v>0</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="39.950000000000003" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>33</v>
@@ -1213,13 +1320,13 @@
         <v>3</v>
       </c>
       <c r="D9" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E9" s="5" t="s">
-        <v>59</v>
-      </c>
       <c r="F9" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
@@ -1234,225 +1341,225 @@
         <v>0</v>
       </c>
       <c r="O9" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="39.950000000000003" customHeight="1">
+      <c r="A10" s="6" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
+      <c r="B10" s="6" t="s">
         <v>61</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>62</v>
       </c>
       <c r="C10" s="6">
         <v>1</v>
       </c>
       <c r="D10" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E10" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="F10" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="G10" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="H10" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="I10" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="J10" s="7">
         <v>80</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="N10" s="7">
         <v>40</v>
       </c>
       <c r="O10" s="7"/>
     </row>
-    <row r="11" spans="1:15" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="39.950000000000003" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C11" s="6">
         <v>1</v>
       </c>
       <c r="D11" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="F11" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="F11" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>73</v>
-      </c>
       <c r="H11" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="I11" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="J11" s="7">
         <v>60</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="N11" s="7">
         <v>30</v>
       </c>
       <c r="O11" s="7"/>
     </row>
-    <row r="12" spans="1:15" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="39.950000000000003" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C12" s="6">
         <v>2</v>
       </c>
       <c r="D12" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E12" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="F12" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G12" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="F12" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="G12" s="7" t="s">
+      <c r="H12" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="I12" s="7" t="s">
         <v>78</v>
-      </c>
-      <c r="I12" s="7" t="s">
-        <v>79</v>
       </c>
       <c r="J12" s="7">
         <v>80</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L12" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="M12" s="7" t="s">
         <v>78</v>
-      </c>
-      <c r="M12" s="7" t="s">
-        <v>79</v>
       </c>
       <c r="N12" s="7">
         <v>60</v>
       </c>
       <c r="O12" s="7"/>
     </row>
-    <row r="13" spans="1:15" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" ht="39.950000000000003" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C13" s="6">
         <v>2</v>
       </c>
       <c r="D13" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E13" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="F13" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G13" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="F13" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>83</v>
-      </c>
       <c r="H13" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="I13" s="7" t="s">
         <v>78</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>79</v>
       </c>
       <c r="J13" s="7">
         <v>50</v>
       </c>
       <c r="K13" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="M13" s="7" t="s">
         <v>84</v>
-      </c>
-      <c r="L13" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="M13" s="7" t="s">
-        <v>85</v>
       </c>
       <c r="N13" s="7">
         <v>65</v>
       </c>
       <c r="O13" s="7"/>
     </row>
-    <row r="14" spans="1:15" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="39.950000000000003" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C14" s="6">
         <v>3</v>
       </c>
       <c r="D14" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E14" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="F14" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G14" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="F14" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="G14" s="7" t="s">
+      <c r="H14" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="I14" s="7" t="s">
         <v>89</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="J14" s="7">
         <v>85</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="M14" s="7"/>
       <c r="N14" s="7">
@@ -1460,42 +1567,42 @@
       </c>
       <c r="O14" s="7"/>
     </row>
-    <row r="15" spans="1:15" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" ht="39.950000000000003" customHeight="1">
       <c r="A15" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C15" s="6">
         <v>3</v>
       </c>
       <c r="D15" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E15" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="F15" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G15" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="F15" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="G15" s="7" t="s">
+      <c r="H15" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="I15" s="7" t="s">
         <v>94</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="I15" s="7" t="s">
-        <v>95</v>
       </c>
       <c r="J15" s="7">
         <v>55</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M15" s="7"/>
       <c r="N15" s="7">
@@ -1503,114 +1610,114 @@
       </c>
       <c r="O15" s="7"/>
     </row>
-    <row r="16" spans="1:15" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" ht="39.950000000000003" customHeight="1">
       <c r="A16" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C16" s="6">
         <v>3</v>
       </c>
       <c r="D16" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E16" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="F16" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G16" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="F16" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>99</v>
-      </c>
       <c r="H16" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="I16" s="7" t="s">
         <v>89</v>
-      </c>
-      <c r="I16" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="J16" s="7">
         <v>75</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="N16" s="7">
         <v>40</v>
       </c>
       <c r="O16" s="7"/>
     </row>
-    <row r="17" spans="1:15" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" ht="39.950000000000003" customHeight="1">
       <c r="A17" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C17" s="6">
         <v>4</v>
       </c>
       <c r="D17" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="E17" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="F17" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G17" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="F17" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>103</v>
-      </c>
       <c r="H17" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J17" s="7">
         <v>60</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="N17" s="7">
         <v>50</v>
       </c>
       <c r="O17" s="7"/>
     </row>
-    <row r="18" spans="1:15" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" ht="39.950000000000003" customHeight="1">
       <c r="A18" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C18" s="6">
         <v>4</v>
       </c>
       <c r="D18" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="E18" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>106</v>
-      </c>
       <c r="F18" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
@@ -1625,27 +1732,27 @@
         <v>0</v>
       </c>
       <c r="O18" s="7" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15">
       <c r="A19" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C19" s="6">
         <v>4</v>
       </c>
       <c r="D19" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E19" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="E19" s="7" t="s">
-        <v>109</v>
-      </c>
       <c r="F19" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G19" s="7"/>
       <c r="H19" s="7"/>
@@ -1660,7 +1767,7 @@
         <v>0</v>
       </c>
       <c r="O19" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[로직] 곰순이 동행 상태 _isGomsuniCompanion 플래그 추가 및 ResultType 정리
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/CBASpecialEvent.xlsx
+++ b/JsonConverter/ExcelFiles/CBASpecialEvent.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GameProjects\CBA\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22D582F9-937A-406C-811F-3C6080C3C6CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50E8509C-6DA2-4EBF-9A2F-E0DE98B28F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -343,9 +343,6 @@
   </si>
   <si>
     <t>네! 함께 모험해요!</t>
-  </si>
-  <si>
-    <t>Companion</t>
   </si>
   <si>
     <t>...안녕히 가세요.</t>
@@ -484,6 +481,10 @@
       </rPr>
       <t>\n넌 살 좀 빼야돼~</t>
     </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Success</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -610,7 +611,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -637,6 +638,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1109,10 +1113,10 @@
         <v>1</v>
       </c>
       <c r="D4" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>109</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>110</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>34</v>
@@ -1731,8 +1735,8 @@
       <c r="N18" s="7">
         <v>0</v>
       </c>
-      <c r="O18" s="7" t="s">
-        <v>106</v>
+      <c r="O18" s="10" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:15">
@@ -1746,10 +1750,10 @@
         <v>4</v>
       </c>
       <c r="D19" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E19" s="7" t="s">
         <v>107</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>108</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>64</v>

</xml_diff>

<commit_message>
[데이터드리븐] CBASpecialEvent ResultText 컬럼 추가 및 JSON 변환
[Logic] 특별 이벤트 결과 텍스트 출력 연결
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/CBASpecialEvent.xlsx
+++ b/JsonConverter/ExcelFiles/CBASpecialEvent.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GameProjects\CBA\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50E8509C-6DA2-4EBF-9A2F-E0DE98B28F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83E9EB97-20D6-4430-A215-D8B2820CB1EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="117">
   <si>
     <t>ID</t>
   </si>
@@ -141,9 +141,6 @@
     <t>bee_step2_b</t>
   </si>
   <si>
-    <t>맞서 싸운다</t>
-  </si>
-  <si>
     <t>bee_step2_c</t>
   </si>
   <si>
@@ -213,18 +210,9 @@
     <t>Gomsuni</t>
   </si>
   <si>
-    <t>어? 아까 그 모자 잡아준 곰이잖아요!</t>
-  </si>
-  <si>
-    <t>고마워요~ 덕분에 찾았어요! 혹시 어디 가세요?</t>
-  </si>
-  <si>
     <t>BG_Meadow</t>
   </si>
   <si>
-    <t>같이 가자고 한다</t>
-  </si>
-  <si>
     <t>gomsuni_step2_a</t>
   </si>
   <si>
@@ -237,24 +225,12 @@
     <t>gomsuni_step1_hat_fail</t>
   </si>
   <si>
-    <t>어머, 아까 그 모자 낚아채려던 곰이잖아요?</t>
-  </si>
-  <si>
-    <t>괜찮아요, 모자는 찾았어요. 근데... 다친 건 아니에요?</t>
-  </si>
-  <si>
     <t>부끄럽지만 말을 건넨다</t>
   </si>
   <si>
     <t>아무렇지 않은 척 지나친다</t>
   </si>
   <si>
-    <t>같이 꿀 먹을래요?</t>
-  </si>
-  <si>
-    <t>정말요? 좋아요!</t>
-  </si>
-  <si>
     <t>꿀을 나눠준다</t>
   </si>
   <si>
@@ -264,9 +240,6 @@
     <t>gomsuni_step3_b</t>
   </si>
   <si>
-    <t>꽃다발을 만든다</t>
-  </si>
-  <si>
     <t>저... 저기요...</t>
   </si>
   <si>
@@ -276,18 +249,9 @@
     <t>용기내어 손을 내민다</t>
   </si>
   <si>
-    <t>엉뚱한 춤을 춘다</t>
-  </si>
-  <si>
     <t>gomsuni_step3_c</t>
   </si>
   <si>
-    <t>같이 놀래요?</t>
-  </si>
-  <si>
-    <t>네! 저도 모험 가고 싶었어요!</t>
-  </si>
-  <si>
     <t>함께 가자고 한다</t>
   </si>
   <si>
@@ -297,24 +261,15 @@
     <t>gomsuni_step4_b</t>
   </si>
   <si>
-    <t>내일 또 만나자고 한다</t>
-  </si>
-  <si>
     <t>으음...</t>
   </si>
   <si>
     <t>저... 괜찮으세요?</t>
   </si>
   <si>
-    <t>다시 용기 낸다</t>
-  </si>
-  <si>
     <t>gomsuni_step4_fail</t>
   </si>
   <si>
-    <t>포기한다</t>
-  </si>
-  <si>
     <t>같이 춤출래요?</t>
   </si>
   <si>
@@ -333,22 +288,35 @@
     <t>음... 글쎄요...</t>
   </si>
   <si>
-    <t>진심을 고백한다</t>
-  </si>
-  <si>
-    <t>특기를 보여준다</t>
-  </si>
-  <si>
-    <t>같이 가요, 곰순이!</t>
-  </si>
-  <si>
-    <t>네! 함께 모험해요!</t>
-  </si>
-  <si>
     <t>...안녕히 가세요.</t>
   </si>
   <si>
-    <t>또 만나요~ (손흔들며 떠남)</t>
+    <t>Success</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>결과텍스트</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>ResultText</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>벌끔이를 물리쳤따!!! 흥, 저 자식은 얼굴만 반반해서 약해빠졌다니까~</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>꿀을 빼앗기고 말았따… 흑흑흑… 저 녀석은 얼굴도 잘생겼으면서 왜 힘도 센거야…. 으허헉…ㅠㅠ</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>곰순씨… 돌아와요오오오오….... 으흐흐흫ㄱ…...</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>예쁜 곰순씨가 나와 동행하기로 했다! 크윽… 너무 행복해…… 지금 난 이 세상 최고의 곰!!</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -385,6 +353,24 @@
       </rPr>
       <t>!!</t>
     </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>어떡하지!!</t>
+    </r>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
@@ -395,6 +381,81 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
+      <t>용감하게 맞서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>싸운다</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>(어…</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>어.. 엄청 예쁜 곰순씨다…</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="3"/>
+      </rPr>
+      <t>…</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>으헤헿,,,)</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
       <t>야</t>
     </r>
     <r>
@@ -479,12 +540,1152 @@
         <rFont val="Arial Unicode MS"/>
         <family val="2"/>
       </rPr>
-      <t>\n넌 살 좀 빼야돼~</t>
+      <t>\n</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>넌</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>살</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>좀</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>빼야돼</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>~</t>
     </r>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>Success</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>고마워요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">~ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>덕분에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>찾았어요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>!\n</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>혹시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>어디</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>가세요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>?</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>(아이쒸…</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>예쁜 곰순씨 모자였잖아?!</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="3"/>
+      </rPr>
+      <t>\n</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>쪽팔리게…</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㅠㅠ)</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>괜찮아요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>모자는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>찾았어요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.\n</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>근데</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">… </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>다친</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>건</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>아니에요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>?</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>요 앞에… 혹시 같이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>가실래요?(두근)</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>같이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>꿀</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>먹을래요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>두근)</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>정말요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">? </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>좋아요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>!</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve"> ^---^</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>꽃다발을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>건넨다(급발진)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>원래 남자는 직진이야</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>엉뚱한</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>춤을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>추며 다가간다</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>같이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>놀래요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>?</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>네</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">! </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>저도</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>모험</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>가고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>싶었어요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>!</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>그냥 내일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>또</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>만나자고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>한다(부끄러워라)</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>다시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">한번 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>용기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>낸다</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>포기한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>저런 미녀는 나에게 어울리지 않아…</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>진심을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>고백한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>우어어어!!!)</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>특기를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>보여준다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>트월킹)</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>같이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>가요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>곰순씨!!!!</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>!</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>네</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">! </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>함께</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>모험해요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>!</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>헤헤</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>~</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>우리 또</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>만나지 말아요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>~ (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>흥 뭐야 진짜;;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>)</t>
+    </r>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -492,7 +1693,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -548,6 +1749,36 @@
       <sz val="10"/>
       <name val="Arial Unicode MS"/>
       <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
       <charset val="129"/>
     </font>
   </fonts>
@@ -611,7 +1842,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -641,6 +1872,24 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -945,23 +2194,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="11.5" customWidth="1"/>
+    <col min="3" max="3" width="9.5" customWidth="1"/>
     <col min="4" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="6" max="6" width="11.625" customWidth="1"/>
     <col min="7" max="7" width="22" customWidth="1"/>
     <col min="8" max="9" width="26" customWidth="1"/>
     <col min="10" max="10" width="10" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
     <col min="12" max="13" width="26" customWidth="1"/>
     <col min="14" max="14" width="10" customWidth="1"/>
-    <col min="15" max="15" width="14" customWidth="1"/>
+    <col min="15" max="16" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="21.95" customHeight="1">
+    <row r="1" spans="1:16" ht="21.95" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1007,8 +2257,11 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" s="11" t="s">
+        <v>89</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" ht="18" customHeight="1">
+    <row r="2" spans="1:16" ht="18" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
@@ -1054,8 +2307,11 @@
       <c r="O2" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="P2" s="2" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="3" spans="1:15" ht="21.95" customHeight="1">
+    <row r="3" spans="1:16" ht="21.95" customHeight="1">
       <c r="A3" s="3" t="s">
         <v>17</v>
       </c>
@@ -1101,8 +2357,11 @@
       <c r="O3" s="3" t="s">
         <v>31</v>
       </c>
+      <c r="P3" s="12" t="s">
+        <v>90</v>
+      </c>
     </row>
-    <row r="4" spans="1:15" ht="39.950000000000003" customHeight="1">
+    <row r="4" spans="1:16" ht="39.950000000000003" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>32</v>
       </c>
@@ -1113,10 +2372,10 @@
         <v>1</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>34</v>
@@ -1133,11 +2392,11 @@
       <c r="J4" s="5">
         <v>60</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="K4" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="M4" s="5" t="s">
         <v>37</v>
@@ -1146,8 +2405,9 @@
         <v>40</v>
       </c>
       <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
     </row>
-    <row r="5" spans="1:15" ht="39.950000000000003" customHeight="1">
+    <row r="5" spans="1:16" ht="39.950000000000003" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>36</v>
       </c>
@@ -1158,39 +2418,40 @@
         <v>2</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>41</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>34</v>
       </c>
       <c r="G5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>42</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>43</v>
       </c>
       <c r="I5" s="5"/>
       <c r="J5" s="5">
         <v>70</v>
       </c>
       <c r="K5" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="M5" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="L5" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="M5" s="5" t="s">
-        <v>45</v>
       </c>
       <c r="N5" s="5">
         <v>50</v>
       </c>
       <c r="O5" s="5"/>
+      <c r="P5" s="5"/>
     </row>
-    <row r="6" spans="1:15" ht="39.950000000000003" customHeight="1">
+    <row r="6" spans="1:16" ht="39.950000000000003" customHeight="1">
       <c r="A6" s="4" t="s">
         <v>37</v>
       </c>
@@ -1201,41 +2462,42 @@
         <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>46</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>47</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>34</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J6" s="5">
         <v>40</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="M6" s="5"/>
       <c r="N6" s="5">
         <v>100</v>
       </c>
       <c r="O6" s="5"/>
+      <c r="P6" s="5"/>
     </row>
-    <row r="7" spans="1:15" ht="39.950000000000003" customHeight="1">
+    <row r="7" spans="1:16" ht="39.950000000000003" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>33</v>
@@ -1244,43 +2506,44 @@
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>51</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>34</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J7" s="5">
         <v>65</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="L7" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N7" s="5">
         <v>50</v>
       </c>
       <c r="O7" s="5"/>
+      <c r="P7" s="5"/>
     </row>
-    <row r="8" spans="1:15" ht="39.950000000000003" customHeight="1">
+    <row r="8" spans="1:16" ht="39.950000000000003" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>33</v>
@@ -1289,10 +2552,10 @@
         <v>3</v>
       </c>
       <c r="D8" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>54</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>55</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>34</v>
@@ -1310,12 +2573,15 @@
         <v>0</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
+      </c>
+      <c r="P8" s="13" t="s">
+        <v>91</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="39.950000000000003" customHeight="1">
+    <row r="9" spans="1:16" ht="39.950000000000003" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>33</v>
@@ -1324,10 +2590,10 @@
         <v>3</v>
       </c>
       <c r="D9" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>57</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>58</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>34</v>
@@ -1345,383 +2611,394 @@
         <v>0</v>
       </c>
       <c r="O9" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="P9" s="13" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="39.950000000000003" customHeight="1">
+      <c r="A10" s="6" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" ht="39.950000000000003" customHeight="1">
-      <c r="A10" s="6" t="s">
+      <c r="B10" s="6" t="s">
         <v>60</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>61</v>
       </c>
       <c r="C10" s="6">
         <v>1</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="H10" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="I10" s="7" t="s">
         <v>63</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>67</v>
       </c>
       <c r="J10" s="7">
         <v>80</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="N10" s="7">
         <v>40</v>
       </c>
       <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
     </row>
-    <row r="11" spans="1:15" ht="39.950000000000003" customHeight="1">
+    <row r="11" spans="1:16" ht="39.950000000000003" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C11" s="6">
         <v>1</v>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>71</v>
+      <c r="D11" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>101</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="J11" s="7">
         <v>60</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="N11" s="7">
         <v>30</v>
       </c>
       <c r="O11" s="7"/>
+      <c r="P11" s="7"/>
     </row>
-    <row r="12" spans="1:15" ht="39.950000000000003" customHeight="1">
+    <row r="12" spans="1:16" ht="39.950000000000003" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C12" s="6">
         <v>2</v>
       </c>
-      <c r="D12" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>75</v>
+      <c r="D12" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>104</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="J12" s="7">
         <v>80</v>
       </c>
-      <c r="K12" s="7" t="s">
-        <v>79</v>
+      <c r="K12" s="16" t="s">
+        <v>105</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="M12" s="7" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="N12" s="7">
         <v>60</v>
       </c>
       <c r="O12" s="7"/>
+      <c r="P12" s="7"/>
     </row>
-    <row r="13" spans="1:15" ht="39.950000000000003" customHeight="1">
+    <row r="13" spans="1:16" ht="39.950000000000003" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C13" s="6">
         <v>2</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="J13" s="7">
         <v>50</v>
       </c>
-      <c r="K13" s="7" t="s">
-        <v>83</v>
+      <c r="K13" s="16" t="s">
+        <v>106</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="N13" s="7">
         <v>65</v>
       </c>
       <c r="O13" s="7"/>
+      <c r="P13" s="7"/>
     </row>
-    <row r="14" spans="1:15" ht="39.950000000000003" customHeight="1">
+    <row r="14" spans="1:16" ht="39.950000000000003" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C14" s="6">
         <v>3</v>
       </c>
-      <c r="D14" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>86</v>
+      <c r="D14" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>108</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="J14" s="7">
         <v>85</v>
       </c>
-      <c r="K14" s="7" t="s">
-        <v>90</v>
+      <c r="K14" s="16" t="s">
+        <v>109</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="M14" s="7"/>
       <c r="N14" s="7">
         <v>50</v>
       </c>
       <c r="O14" s="7"/>
+      <c r="P14" s="7"/>
     </row>
-    <row r="15" spans="1:15" ht="39.950000000000003" customHeight="1">
+    <row r="15" spans="1:16" ht="39.950000000000003" customHeight="1">
       <c r="A15" s="6" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C15" s="6">
         <v>3</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>93</v>
+        <v>61</v>
+      </c>
+      <c r="G15" s="16" t="s">
+        <v>110</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="J15" s="7">
         <v>55</v>
       </c>
-      <c r="K15" s="7" t="s">
-        <v>95</v>
+      <c r="K15" s="16" t="s">
+        <v>111</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="M15" s="7"/>
       <c r="N15" s="7">
         <v>100</v>
       </c>
       <c r="O15" s="7"/>
+      <c r="P15" s="7"/>
     </row>
-    <row r="16" spans="1:15" ht="39.950000000000003" customHeight="1">
+    <row r="16" spans="1:16" ht="39.950000000000003" customHeight="1">
       <c r="A16" s="6" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C16" s="6">
         <v>3</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="J16" s="7">
         <v>75</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="N16" s="7">
         <v>40</v>
       </c>
       <c r="O16" s="7"/>
+      <c r="P16" s="7"/>
     </row>
-    <row r="17" spans="1:15" ht="39.950000000000003" customHeight="1">
+    <row r="17" spans="1:16" ht="39.950000000000003" customHeight="1">
       <c r="A17" s="6" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C17" s="6">
         <v>4</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>102</v>
+        <v>61</v>
+      </c>
+      <c r="G17" s="16" t="s">
+        <v>112</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="J17" s="7">
         <v>60</v>
       </c>
-      <c r="K17" s="7" t="s">
-        <v>103</v>
+      <c r="K17" s="16" t="s">
+        <v>113</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="N17" s="7">
         <v>50</v>
       </c>
       <c r="O17" s="7"/>
+      <c r="P17" s="7"/>
     </row>
-    <row r="18" spans="1:15" ht="39.950000000000003" customHeight="1">
+    <row r="18" spans="1:16" ht="39.950000000000003" customHeight="1">
       <c r="A18" s="6" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C18" s="6">
         <v>4</v>
       </c>
-      <c r="D18" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>105</v>
+      <c r="D18" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="E18" s="16" t="s">
+        <v>115</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
@@ -1736,27 +3013,30 @@
         <v>0</v>
       </c>
       <c r="O18" s="10" t="s">
-        <v>110</v>
+        <v>88</v>
+      </c>
+      <c r="P18" s="14" t="s">
+        <v>94</v>
       </c>
     </row>
-    <row r="19" spans="1:15">
+    <row r="19" spans="1:16" ht="40.5">
       <c r="A19" s="6" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C19" s="6">
         <v>4</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>107</v>
+        <v>87</v>
+      </c>
+      <c r="E19" s="16" t="s">
+        <v>116</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G19" s="7"/>
       <c r="H19" s="7"/>
@@ -1771,7 +3051,10 @@
         <v>0</v>
       </c>
       <c r="O19" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
+      </c>
+      <c r="P19" s="15" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>